<commit_message>
PA12: ajustes importação + planilhas unificadas
- import_doc_status: mapeia Apto=1, Inapto=2, Não se aplica=3 (era só Apto=1)
- Funcionários: lê colunas 26-27 → integracao_corsan e sertras na importação
- Funcionários: INSERT/UPDATE/docMap incluem integracao_corsan e sertras
- Trechos: DN lido como inteiro (não texto formatado)
- Modelos xlsx substituídos pelas planilhas unificadas PA12 (identidade Gravitas,
  listas suspensas, realce automático, aba Instruções, cabeçalho L6 / dados L7)

https://claude.ai/code/session_01GB592wHtRegLJEtgwh4ZdP
</commit_message>
<xml_diff>
--- a/painel/assets/modelos/equipamentos-leves.xlsx
+++ b/painel/assets/modelos/equipamentos-leves.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Equipamentos Leves" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modelo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,41 +29,57 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FF1B2A4A"/>
+      <color rgb="00E0A53D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C7D2E5"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00A96C2A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="006B7686"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001E2738"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A2D4F"/>
       <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="FF555555"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="FF555555"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="FF856404"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="FF777777"/>
-      <sz val="10"/>
+      <color rgb="001A2D4F"/>
+      <sz val="12"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -71,37 +88,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE8EDF5"/>
+        <fgColor rgb="001A2D4F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF5F7FA"/>
+        <fgColor rgb="00F6E7CF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFAFAFA"/>
+        <fgColor rgb="00F4F6FA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF3CD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1B2A4A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF155724"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF9C4"/>
+        <fgColor rgb="00FFF7D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -115,44 +117,59 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFD0D0D0"/>
+        <color rgb="00E4E8EF"/>
       </left>
       <right style="thin">
-        <color rgb="FFD0D0D0"/>
+        <color rgb="00E4E8EF"/>
       </right>
       <top style="thin">
-        <color rgb="FFD0D0D0"/>
+        <color rgb="00E4E8EF"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFD0D0D0"/>
+        <color rgb="00E4E8EF"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -228,6 +245,106 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Gravitas</author>
+  </authors>
+  <commentList>
+    <comment ref="A6" authorId="0" shapeId="0">
+      <text>
+        <t>Tipo (ex.: Compactador, Bomba d'água, Placa vibratória).</t>
+      </text>
+    </comment>
+    <comment ref="B6" authorId="0" shapeId="0">
+      <text>
+        <t>Referência/patrimônio (chave). Se vazia, usa Modelo.</t>
+      </text>
+    </comment>
+    <comment ref="C6" authorId="0" shapeId="0">
+      <text>
+        <t>Modelo.</t>
+      </text>
+    </comment>
+    <comment ref="D6" authorId="0" shapeId="0">
+      <text>
+        <t>Ano de fabricação (número inteiro).</t>
+      </text>
+    </comment>
+    <comment ref="E6" authorId="0" shapeId="0">
+      <text>
+        <t>Proprietário.</t>
+      </text>
+    </comment>
+    <comment ref="F6" authorId="0" shapeId="0">
+      <text>
+        <t>Combustível (lista).</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="666750" cy="666750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="419100" cy="419100"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -519,116 +636,864 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>MODELO — IMPORTAÇÃO DE EQUIPAMENTOS LEVES</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Preencha a partir da linha 7.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>🟢 Colunas com fundo verde são OBRIGATÓRIAS  |  Demais colunas são opcionais  |  ⚠️ Não altere as 6 primeiras linhas</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Referência é a chave única (ex: placa ou código). Se vazia, Modelo será usado como chave.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="8" customHeight="1"/>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>GRAVITAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>PAINEL DE CONTROLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Equipamentos Leves  ·  Modelo de Importação</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>⚠  NÃO altere as linhas 1 a 6. Cabeçalho na linha 6. Preencha a partir da LINHA 7, somente as células em amarelo claro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Listas (▾): escolha o valor. Datas DD/MM/AAAA. Decimais com vírgula. Ano = inteiro. CPF só números. Passe o mouse no título (▾) para ajuda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Referência</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Modelo</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Ano</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Proprietário</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>Combustível</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Caminhonete</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>ABC-1234</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Hilux 2023</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>2023</v>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Gravitas</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>Diesel</t>
-        </is>
-      </c>
+    <row r="7">
+      <c r="A7" s="8" t="n"/>
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="8" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="n"/>
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="8" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="8" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="8" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="8" t="n"/>
+      <c r="F12" s="8" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="8" t="n"/>
+      <c r="F13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="9" t="n"/>
+      <c r="E14" s="8" t="n"/>
+      <c r="F14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n"/>
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="8" t="n"/>
+      <c r="F15" s="8" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n"/>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="9" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n"/>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="9" t="n"/>
+      <c r="E18" s="8" t="n"/>
+      <c r="F18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="9" t="n"/>
+      <c r="E19" s="8" t="n"/>
+      <c r="F19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="9" t="n"/>
+      <c r="E20" s="8" t="n"/>
+      <c r="F20" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n"/>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="9" t="n"/>
+      <c r="E21" s="8" t="n"/>
+      <c r="F21" s="8" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="8" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n"/>
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="8" t="n"/>
+      <c r="F23" s="8" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n"/>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="9" t="n"/>
+      <c r="E24" s="8" t="n"/>
+      <c r="F24" s="8" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="n"/>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="8" t="n"/>
+      <c r="F25" s="8" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="8" t="n"/>
+      <c r="F26" s="8" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="8" t="n"/>
+      <c r="F27" s="8" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="9" t="n"/>
+      <c r="E28" s="8" t="n"/>
+      <c r="F28" s="8" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="n"/>
+      <c r="B29" s="8" t="n"/>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="8" t="n"/>
+      <c r="F29" s="8" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="n"/>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="9" t="n"/>
+      <c r="E30" s="8" t="n"/>
+      <c r="F30" s="8" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n"/>
+      <c r="B31" s="8" t="n"/>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="9" t="n"/>
+      <c r="E31" s="8" t="n"/>
+      <c r="F31" s="8" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n"/>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="9" t="n"/>
+      <c r="E32" s="8" t="n"/>
+      <c r="F32" s="8" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="n"/>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="9" t="n"/>
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="8" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n"/>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="8" t="n"/>
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="8" t="n"/>
+      <c r="F34" s="8" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="n"/>
+      <c r="B35" s="8" t="n"/>
+      <c r="C35" s="8" t="n"/>
+      <c r="D35" s="9" t="n"/>
+      <c r="E35" s="8" t="n"/>
+      <c r="F35" s="8" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n"/>
+      <c r="B36" s="8" t="n"/>
+      <c r="C36" s="8" t="n"/>
+      <c r="D36" s="9" t="n"/>
+      <c r="E36" s="8" t="n"/>
+      <c r="F36" s="8" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="n"/>
+      <c r="B37" s="8" t="n"/>
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="9" t="n"/>
+      <c r="E37" s="8" t="n"/>
+      <c r="F37" s="8" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n"/>
+      <c r="B38" s="8" t="n"/>
+      <c r="C38" s="8" t="n"/>
+      <c r="D38" s="9" t="n"/>
+      <c r="E38" s="8" t="n"/>
+      <c r="F38" s="8" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n"/>
+      <c r="B39" s="8" t="n"/>
+      <c r="C39" s="8" t="n"/>
+      <c r="D39" s="9" t="n"/>
+      <c r="E39" s="8" t="n"/>
+      <c r="F39" s="8" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="n"/>
+      <c r="B40" s="8" t="n"/>
+      <c r="C40" s="8" t="n"/>
+      <c r="D40" s="9" t="n"/>
+      <c r="E40" s="8" t="n"/>
+      <c r="F40" s="8" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="n"/>
+      <c r="B41" s="8" t="n"/>
+      <c r="C41" s="8" t="n"/>
+      <c r="D41" s="9" t="n"/>
+      <c r="E41" s="8" t="n"/>
+      <c r="F41" s="8" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n"/>
+      <c r="B42" s="8" t="n"/>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="9" t="n"/>
+      <c r="E42" s="8" t="n"/>
+      <c r="F42" s="8" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="n"/>
+      <c r="B43" s="8" t="n"/>
+      <c r="C43" s="8" t="n"/>
+      <c r="D43" s="9" t="n"/>
+      <c r="E43" s="8" t="n"/>
+      <c r="F43" s="8" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n"/>
+      <c r="B44" s="8" t="n"/>
+      <c r="C44" s="8" t="n"/>
+      <c r="D44" s="9" t="n"/>
+      <c r="E44" s="8" t="n"/>
+      <c r="F44" s="8" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="n"/>
+      <c r="B45" s="8" t="n"/>
+      <c r="C45" s="8" t="n"/>
+      <c r="D45" s="9" t="n"/>
+      <c r="E45" s="8" t="n"/>
+      <c r="F45" s="8" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="n"/>
+      <c r="B46" s="8" t="n"/>
+      <c r="C46" s="8" t="n"/>
+      <c r="D46" s="9" t="n"/>
+      <c r="E46" s="8" t="n"/>
+      <c r="F46" s="8" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="n"/>
+      <c r="B47" s="8" t="n"/>
+      <c r="C47" s="8" t="n"/>
+      <c r="D47" s="9" t="n"/>
+      <c r="E47" s="8" t="n"/>
+      <c r="F47" s="8" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="n"/>
+      <c r="B48" s="8" t="n"/>
+      <c r="C48" s="8" t="n"/>
+      <c r="D48" s="9" t="n"/>
+      <c r="E48" s="8" t="n"/>
+      <c r="F48" s="8" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="n"/>
+      <c r="B49" s="8" t="n"/>
+      <c r="C49" s="8" t="n"/>
+      <c r="D49" s="9" t="n"/>
+      <c r="E49" s="8" t="n"/>
+      <c r="F49" s="8" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="n"/>
+      <c r="B50" s="8" t="n"/>
+      <c r="C50" s="8" t="n"/>
+      <c r="D50" s="9" t="n"/>
+      <c r="E50" s="8" t="n"/>
+      <c r="F50" s="8" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="n"/>
+      <c r="B51" s="8" t="n"/>
+      <c r="C51" s="8" t="n"/>
+      <c r="D51" s="9" t="n"/>
+      <c r="E51" s="8" t="n"/>
+      <c r="F51" s="8" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="n"/>
+      <c r="B52" s="8" t="n"/>
+      <c r="C52" s="8" t="n"/>
+      <c r="D52" s="9" t="n"/>
+      <c r="E52" s="8" t="n"/>
+      <c r="F52" s="8" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="n"/>
+      <c r="B53" s="8" t="n"/>
+      <c r="C53" s="8" t="n"/>
+      <c r="D53" s="9" t="n"/>
+      <c r="E53" s="8" t="n"/>
+      <c r="F53" s="8" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="n"/>
+      <c r="B54" s="8" t="n"/>
+      <c r="C54" s="8" t="n"/>
+      <c r="D54" s="9" t="n"/>
+      <c r="E54" s="8" t="n"/>
+      <c r="F54" s="8" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="n"/>
+      <c r="B55" s="8" t="n"/>
+      <c r="C55" s="8" t="n"/>
+      <c r="D55" s="9" t="n"/>
+      <c r="E55" s="8" t="n"/>
+      <c r="F55" s="8" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="n"/>
+      <c r="B56" s="8" t="n"/>
+      <c r="C56" s="8" t="n"/>
+      <c r="D56" s="9" t="n"/>
+      <c r="E56" s="8" t="n"/>
+      <c r="F56" s="8" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="n"/>
+      <c r="B57" s="8" t="n"/>
+      <c r="C57" s="8" t="n"/>
+      <c r="D57" s="9" t="n"/>
+      <c r="E57" s="8" t="n"/>
+      <c r="F57" s="8" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="n"/>
+      <c r="B58" s="8" t="n"/>
+      <c r="C58" s="8" t="n"/>
+      <c r="D58" s="9" t="n"/>
+      <c r="E58" s="8" t="n"/>
+      <c r="F58" s="8" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="n"/>
+      <c r="B59" s="8" t="n"/>
+      <c r="C59" s="8" t="n"/>
+      <c r="D59" s="9" t="n"/>
+      <c r="E59" s="8" t="n"/>
+      <c r="F59" s="8" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="n"/>
+      <c r="B60" s="8" t="n"/>
+      <c r="C60" s="8" t="n"/>
+      <c r="D60" s="9" t="n"/>
+      <c r="E60" s="8" t="n"/>
+      <c r="F60" s="8" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="n"/>
+      <c r="B61" s="8" t="n"/>
+      <c r="C61" s="8" t="n"/>
+      <c r="D61" s="9" t="n"/>
+      <c r="E61" s="8" t="n"/>
+      <c r="F61" s="8" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="n"/>
+      <c r="B62" s="8" t="n"/>
+      <c r="C62" s="8" t="n"/>
+      <c r="D62" s="9" t="n"/>
+      <c r="E62" s="8" t="n"/>
+      <c r="F62" s="8" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="n"/>
+      <c r="B63" s="8" t="n"/>
+      <c r="C63" s="8" t="n"/>
+      <c r="D63" s="9" t="n"/>
+      <c r="E63" s="8" t="n"/>
+      <c r="F63" s="8" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="n"/>
+      <c r="B64" s="8" t="n"/>
+      <c r="C64" s="8" t="n"/>
+      <c r="D64" s="9" t="n"/>
+      <c r="E64" s="8" t="n"/>
+      <c r="F64" s="8" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="n"/>
+      <c r="B65" s="8" t="n"/>
+      <c r="C65" s="8" t="n"/>
+      <c r="D65" s="9" t="n"/>
+      <c r="E65" s="8" t="n"/>
+      <c r="F65" s="8" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="n"/>
+      <c r="B66" s="8" t="n"/>
+      <c r="C66" s="8" t="n"/>
+      <c r="D66" s="9" t="n"/>
+      <c r="E66" s="8" t="n"/>
+      <c r="F66" s="8" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="n"/>
+      <c r="B67" s="8" t="n"/>
+      <c r="C67" s="8" t="n"/>
+      <c r="D67" s="9" t="n"/>
+      <c r="E67" s="8" t="n"/>
+      <c r="F67" s="8" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="n"/>
+      <c r="B68" s="8" t="n"/>
+      <c r="C68" s="8" t="n"/>
+      <c r="D68" s="9" t="n"/>
+      <c r="E68" s="8" t="n"/>
+      <c r="F68" s="8" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="n"/>
+      <c r="B69" s="8" t="n"/>
+      <c r="C69" s="8" t="n"/>
+      <c r="D69" s="9" t="n"/>
+      <c r="E69" s="8" t="n"/>
+      <c r="F69" s="8" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="n"/>
+      <c r="B70" s="8" t="n"/>
+      <c r="C70" s="8" t="n"/>
+      <c r="D70" s="9" t="n"/>
+      <c r="E70" s="8" t="n"/>
+      <c r="F70" s="8" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="n"/>
+      <c r="B71" s="8" t="n"/>
+      <c r="C71" s="8" t="n"/>
+      <c r="D71" s="9" t="n"/>
+      <c r="E71" s="8" t="n"/>
+      <c r="F71" s="8" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="n"/>
+      <c r="B72" s="8" t="n"/>
+      <c r="C72" s="8" t="n"/>
+      <c r="D72" s="9" t="n"/>
+      <c r="E72" s="8" t="n"/>
+      <c r="F72" s="8" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="n"/>
+      <c r="B73" s="8" t="n"/>
+      <c r="C73" s="8" t="n"/>
+      <c r="D73" s="9" t="n"/>
+      <c r="E73" s="8" t="n"/>
+      <c r="F73" s="8" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="n"/>
+      <c r="B74" s="8" t="n"/>
+      <c r="C74" s="8" t="n"/>
+      <c r="D74" s="9" t="n"/>
+      <c r="E74" s="8" t="n"/>
+      <c r="F74" s="8" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="n"/>
+      <c r="B75" s="8" t="n"/>
+      <c r="C75" s="8" t="n"/>
+      <c r="D75" s="9" t="n"/>
+      <c r="E75" s="8" t="n"/>
+      <c r="F75" s="8" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="8" t="n"/>
+      <c r="B76" s="8" t="n"/>
+      <c r="C76" s="8" t="n"/>
+      <c r="D76" s="9" t="n"/>
+      <c r="E76" s="8" t="n"/>
+      <c r="F76" s="8" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="n"/>
+      <c r="B77" s="8" t="n"/>
+      <c r="C77" s="8" t="n"/>
+      <c r="D77" s="9" t="n"/>
+      <c r="E77" s="8" t="n"/>
+      <c r="F77" s="8" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="8" t="n"/>
+      <c r="B78" s="8" t="n"/>
+      <c r="C78" s="8" t="n"/>
+      <c r="D78" s="9" t="n"/>
+      <c r="E78" s="8" t="n"/>
+      <c r="F78" s="8" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="n"/>
+      <c r="B79" s="8" t="n"/>
+      <c r="C79" s="8" t="n"/>
+      <c r="D79" s="9" t="n"/>
+      <c r="E79" s="8" t="n"/>
+      <c r="F79" s="8" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="8" t="n"/>
+      <c r="B80" s="8" t="n"/>
+      <c r="C80" s="8" t="n"/>
+      <c r="D80" s="9" t="n"/>
+      <c r="E80" s="8" t="n"/>
+      <c r="F80" s="8" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="8" t="n"/>
+      <c r="B81" s="8" t="n"/>
+      <c r="C81" s="8" t="n"/>
+      <c r="D81" s="9" t="n"/>
+      <c r="E81" s="8" t="n"/>
+      <c r="F81" s="8" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="n"/>
+      <c r="B82" s="8" t="n"/>
+      <c r="C82" s="8" t="n"/>
+      <c r="D82" s="9" t="n"/>
+      <c r="E82" s="8" t="n"/>
+      <c r="F82" s="8" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="8" t="n"/>
+      <c r="B83" s="8" t="n"/>
+      <c r="C83" s="8" t="n"/>
+      <c r="D83" s="9" t="n"/>
+      <c r="E83" s="8" t="n"/>
+      <c r="F83" s="8" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="8" t="n"/>
+      <c r="B84" s="8" t="n"/>
+      <c r="C84" s="8" t="n"/>
+      <c r="D84" s="9" t="n"/>
+      <c r="E84" s="8" t="n"/>
+      <c r="F84" s="8" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="n"/>
+      <c r="B85" s="8" t="n"/>
+      <c r="C85" s="8" t="n"/>
+      <c r="D85" s="9" t="n"/>
+      <c r="E85" s="8" t="n"/>
+      <c r="F85" s="8" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="8" t="n"/>
+      <c r="B86" s="8" t="n"/>
+      <c r="C86" s="8" t="n"/>
+      <c r="D86" s="9" t="n"/>
+      <c r="E86" s="8" t="n"/>
+      <c r="F86" s="8" t="n"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="1" sort="1" password="D8C7"/>
   <mergeCells count="5">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B2:F2"/>
     <mergeCell ref="A5:F5"/>
+    <mergeCell ref="B3:F3"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="B1:F1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="D7:D86" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Número inválido" error="Use número inteiro (sem vírgula)." type="whole" operator="greaterThan">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="F7:F86" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Escolha um valor da lista." prompt="Combustível (lista)." type="list">
+      <formula1>"Diesel,Gasolina,Elétrico,Outro"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B4:B18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="38" customHeight="1"/>
+    <row r="4">
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>GRAVITAS · PAINEL DE CONTROLE — Equipamentos Leves</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="11" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>• Não altere as linhas de cabeçalho/instruções (1 a 6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>• Preencha só as células em AMARELO CLARO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>• Onde houver lista (▾), escolha um valor — não digite à mão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>• Datas no formato DD/MM/AAAA. Decimais com vírgula. Ano = número inteiro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>• Status de documento: Apto / Inapto / Não se aplica (ou deixe em branco).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Colunas:</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>•  Tipo: Tipo (ex.: Compactador, Bomba d'água, Placa vibratória).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>•  Referência: Referência/patrimônio (chave). Se vazia, usa Modelo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>•  Modelo: Modelo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>•  Ano: Ano de fabricação (número inteiro).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>•  Proprietário: Proprietário.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>•  Combustível: Combustível (lista).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="D8C7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>